<commit_message>
feat(F-NAR-019): TREE-DIF-057 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-057.xlsx
+++ b/stories/arbres/TREE-DIF-057.xlsx
@@ -2726,17 +2726,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>J'attends le dernier trait. Merci, Sarah. Elle compte les rayons sur le verre tiède. Le bocal attend sur la table, sans bouger. La craie s'arrête, pile. Il a son soleil, là. Tu viens, alors ? Oui, j'apporte la craie. Tu as laissé le soleil finir.</t>
+          <t>J'attends le dernier trait. Merci, le verre peut patienter. Sarah pose le bocal comme un second soleil. Elle compte les rayons sur la buée du verre. La craie s'arrête, pile, contre le col. Mon soleil a réveillé le tien. Tu viens, alors ? Oui, j'apporte la craie. Tu as laissé le soleil finir.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'attends le dernier trait. Merci, Sarah. Elle compte les rayons sur le verre tiède. Le bocal attend sur la table, sans bouger. La craie s'arrête, pile. Il a son &lt;emphasis level="moderate"&gt;soleil&lt;/emphasis&gt;, là. Tu viens, alors ? Oui, j'apporte la craie. Tu as laissé le soleil finir.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'attends le dernier trait. Merci, le verre peut patienter. Sarah pose le bocal comme un second &lt;emphasis level="moderate"&gt;soleil&lt;/emphasis&gt;. Elle compte les rayons sur la buée du verre. La craie s'arrête, pile, contre le col. Mon soleil a réveillé le tien. Tu viens, alors ? Oui, j'apporte la craie. Tu as laissé le soleil finir.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>J'attends le dernier trait. Merci, Sarah. Elle compte les rayons sur le verre tiède. Le bocal attend sur la table, sans bouger. La craie s'arrête, pile. Il a son &lt;emphasis&gt;soleil&lt;/emphasis&gt;, là. Tu viens, alors ? Oui, j'apporte la craie. Tu as laissé le soleil finir. [pause]</t>
+          <t>J'attends le dernier trait. Merci, le verre peut patienter. Sarah pose le bocal comme un second &lt;emphasis&gt;soleil&lt;/emphasis&gt;. Elle compte les rayons sur la buée du verre. La craie s'arrête, pile, contre le col. Mon soleil a réveillé le tien. Tu viens, alors ? Oui, j'apporte la craie. Tu as laissé le soleil finir. [pause]</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -2871,11 +2871,11 @@
       <c r="AW10" t="inlineStr">
         <is>
           <t>enfant-f|J'attends le dernier trait.
-copain|Merci, Sarah.
-narrateur|Elle compte les rayons sur le verre tiède.
-narrateur|Le bocal attend sur la table, sans bouger.
-narrateur|La craie s'arrête, pile.
-copain|Il a son soleil, là.
+copain|Merci, le verre peut patienter.
+narrateur|Sarah pose le bocal comme un second soleil.
+narrateur|Elle compte les rayons sur la buée du verre.
+narrateur|La craie s'arrête, pile, contre le col.
+copain|Mon soleil a réveillé le tien.
 enfant-f|Tu viens, alors ?
 copain|Oui, j'apporte la craie.
 papa|Tu as laissé le soleil finir.</t>
@@ -2910,17 +2910,17 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Le soleil de craie reste sur la pierre. Il a son dernier trait, Sarah. Oui, tout jaune. La craie a laissé la place. Le prunier fait un petit toc. Le bocal garde un toc, tiède contre le bois. Nino noue le grelot, les doigts tâchés de jaune. Le jardin chante, là. La poussière jaune dort sur les genoux de Nino.</t>
+          <t>Le soleil de craie chauffe le bois de la table. Il a son dernier trait, Sarah. Oui, bien jaune. La craie a laissé la place. Le prunier fait un petit toc. Le bocal garde un toc, tiède contre le bois. Nino noue le grelot, les doigts tâchés de jaune. Le jardin chante, là. La poussière jaune dort sur les genoux de Nino.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le soleil de craie reste sur la pierre. Il a son dernier trait, Sarah. Oui, tout jaune. La craie a laissé la place. Le &lt;emphasis level="moderate"&gt;prunier&lt;/emphasis&gt; fait un petit toc. Le bocal garde un toc, tiède contre le bois. Nino noue le grelot, les doigts tâchés de jaune. Le jardin chante, là. La poussière jaune dort sur les genoux de Nino.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le soleil de craie chauffe le bois de la table. Il a son dernier trait, Sarah. Oui, bien jaune. La craie a laissé la place. Le &lt;emphasis level="moderate"&gt;prunier&lt;/emphasis&gt; fait un petit toc. Le bocal garde un toc, tiède contre le bois. Nino noue le grelot, les doigts tâchés de jaune. Le jardin chante, là. La poussière jaune dort sur les genoux de Nino.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le soleil de craie reste sur la pierre. Il a son dernier trait, Sarah. Oui, tout jaune. La craie a laissé la place. Le &lt;emphasis&gt;prunier&lt;/emphasis&gt; fait un petit toc. Le bocal garde un toc, tiède contre le bois. Nino noue le grelot, les doigts tâchés de jaune. Le jardin chante, là. La poussière jaune dort sur les genoux de Nino.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le soleil de craie chauffe le bois de la table. Il a son dernier trait, Sarah. Oui, bien jaune. La craie a laissé la place. Le &lt;emphasis&gt;prunier&lt;/emphasis&gt; fait un petit toc. Le bocal garde un toc, tiède contre le bois. Nino noue le grelot, les doigts tâchés de jaune. Le jardin chante, là. La poussière jaune dort sur les genoux de Nino.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -3058,9 +3058,9 @@
       </c>
       <c r="AW11" t="inlineStr">
         <is>
-          <t>narrateur|Le soleil de craie reste sur la pierre.
+          <t>narrateur|Le soleil de craie chauffe le bois de la table.
 copain|Il a son dernier trait, Sarah.
-enfant-f|Oui, tout jaune.
+enfant-f|Oui, bien jaune.
 papa|La craie a laissé la place.
 maman|Le prunier fait un petit toc.
 narrateur|Le bocal garde un toc, tiède contre le bois.
@@ -3098,17 +3098,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Nino, un carillon t'écoute. Elle glisse le bocal contre la craie. Sa voix reste près de lui, presque un souffle. Il a une oreille, lui aussi ? Oui, creuse comme un soleil. Je viens, alors. Il pose la craie, sans la perdre. Tu as parlé contre son dessin. C'est lui qui a dit oui.</t>
+          <t>Nino, le verre a une oreille. Elle glisse le bocal contre le rayon manquant. Sa voix reste un souffle, collée au bois. Il écoute mon soleil, lui aussi ? Oui, creux comme un trait. Je viens, alors. Il pose la craie dans l'ombre du verre. Tu as parlé contre son dessin. C'est lui qui a dit oui.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino, un &lt;emphasis level="moderate"&gt;carillon&lt;/emphasis&gt; t'écoute. Elle glisse le bocal contre la craie. Sa voix reste près de lui, presque un souffle. Il a une oreille, lui aussi ? Oui, creuse comme un soleil. Je viens, alors. Il pose la craie, sans la perdre. Tu as parlé contre son dessin. C'est lui qui a dit oui.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino, le verre a une oreille. Elle glisse le bocal contre le rayon manquant. Sa voix reste un souffle, collée au bois. Il écoute mon soleil, lui aussi ? Oui, creux comme un trait. Je viens, alors. Il pose la craie dans l'ombre du verre. Tu as parlé contre son dessin. C'est lui qui a dit oui.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Nino, un &lt;emphasis&gt;carillon&lt;/emphasis&gt; t'écoute. Elle glisse le bocal contre la craie. Sa voix reste près de lui, presque un souffle. Il a une oreille, lui aussi ? Oui, creuse comme un soleil. Je viens, alors. Il pose la craie, sans la perdre. Tu as parlé contre son dessin. C'est lui qui a dit oui. [pause]</t>
+          <t>Nino, le verre a une oreille. Elle glisse le bocal contre le rayon manquant. Sa voix reste un souffle, collée au bois. Il écoute mon soleil, lui aussi ? Oui, creux comme un trait. Je viens, alors. Il pose la craie dans l'ombre du verre. Tu as parlé contre son dessin. C'est lui qui a dit oui. [pause]</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -3242,13 +3242,13 @@
       </c>
       <c r="AW12" t="inlineStr">
         <is>
-          <t>enfant-f|Nino, un carillon t'écoute.
-narrateur|Elle glisse le bocal contre la craie.
-narrateur|Sa voix reste près de lui, presque un souffle.
-copain|Il a une oreille, lui aussi ?
-enfant-f|Oui, creuse comme un soleil.
+          <t>enfant-f|Nino, le verre a une oreille.
+narrateur|Elle glisse le bocal contre le rayon manquant.
+narrateur|Sa voix reste un souffle, collée au bois.
+copain|Il écoute mon soleil, lui aussi ?
+enfant-f|Oui, creux comme un trait.
 copain|Je viens, alors.
-narrateur|Il pose la craie, sans la perdre.
+narrateur|Il pose la craie dans l'ombre du verre.
 papa|Tu as parlé contre son dessin.
 maman|C'est lui qui a dit oui.</t>
         </is>
@@ -3470,17 +3470,17 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Je m'assois à côté. Sarah s'assoit au pied de la table. Elle ne touche pas la craie. Tu vois le rayon, toi aussi ? Oui, il pique un peu. Un dernier trait les fait souffler. On accroche, après ça. Tu as écouté son soleil. C'est lui qui a dit après.</t>
+          <t>Je m'assois à côté. Sarah s'assoit au pied de la table. Le bocal tient chaud entre eux, sans bouger. Tu vois le rayon, toi aussi ? Oui, il pique un peu. Un dernier trait les fait souffler ensemble. On accroche, après ça. Tu as écouté son soleil. C'est lui qui a dit après.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Je m'assois à &lt;emphasis level="moderate"&gt;côté&lt;/emphasis&gt;. Sarah s'assoit au pied de la table. Elle ne touche pas la craie. Tu vois le rayon, toi aussi ? Oui, il pique un peu. Un dernier trait les fait souffler. On accroche, après ça. Tu as écouté son soleil. C'est lui qui a dit après.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Je m'assois à &lt;emphasis level="moderate"&gt;côté&lt;/emphasis&gt;. Sarah s'assoit au pied de la table. Le bocal tient chaud entre eux, sans bouger. Tu vois le rayon, toi aussi ? Oui, il pique un peu. Un dernier trait les fait souffler ensemble. On accroche, après ça. Tu as écouté son soleil. C'est lui qui a dit après.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Je m'assois à &lt;emphasis&gt;côté&lt;/emphasis&gt;. Sarah s'assoit au pied de la table. Elle ne touche pas la craie. Tu vois le rayon, toi aussi ? Oui, il pique un peu. Un dernier trait les fait souffler. On accroche, après ça. Tu as écouté son soleil. C'est lui qui a dit après. [pause]</t>
+          <t>Je m'assois à &lt;emphasis&gt;côté&lt;/emphasis&gt;. Sarah s'assoit au pied de la table. Le bocal tient chaud entre eux, sans bouger. Tu vois le rayon, toi aussi ? Oui, il pique un peu. Un dernier trait les fait souffler ensemble. On accroche, après ça. Tu as écouté son soleil. C'est lui qui a dit après. [pause]</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -3616,10 +3616,10 @@
         <is>
           <t>enfant-f|Je m'assois à côté.
 narrateur|Sarah s'assoit au pied de la table.
-narrateur|Elle ne touche pas la craie.
+narrateur|Le bocal tient chaud entre eux, sans bouger.
 copain|Tu vois le rayon, toi aussi ?
 enfant-f|Oui, il pique un peu.
-narrateur|Un dernier trait les fait souffler.
+narrateur|Un dernier trait les fait souffler ensemble.
 copain|On accroche, après ça.
 papa|Tu as écouté son soleil.
 maman|C'est lui qui a dit après.</t>
@@ -4227,17 +4227,17 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>J'attends l'envol. Merci, Sarah. La table garde le bocal, sans le bouger. La coccinelle ouvre une aile, puis part. Elle a volé, là. Tu viens, alors ? Oui, je laisse la rose. Tu as laissé la rose finir. Il a dit oui, après.</t>
+          <t>J'attends l'envol. Merci, la rose d'abord. Sarah regarde la rose dans le verre du bocal. La petite bête y marche, à l'envers. Une aile s'ouvre, et l'image s'envole. Elle a volé, là. Tu viens, alors ? Oui, je laisse la rose. Tu as laissé la rose finir.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'attends l'&lt;emphasis level="moderate"&gt;envol&lt;/emphasis&gt;. Merci, Sarah. La table garde le bocal, sans le bouger. La coccinelle ouvre une aile, puis part. Elle a volé, là. Tu viens, alors ? Oui, je laisse la rose. Tu as laissé la rose finir. Il a dit oui, après.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'attends l'&lt;emphasis level="moderate"&gt;envol&lt;/emphasis&gt;. Merci, la rose d'abord. Sarah regarde la rose dans le verre du bocal. La petite bête y marche, à l'envers. Une aile s'ouvre, et l'image s'envole. Elle a volé, là. Tu viens, alors ? Oui, je laisse la rose. Tu as laissé la rose finir.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>J'attends l'&lt;emphasis&gt;envol&lt;/emphasis&gt;. Merci, Sarah. La table garde le bocal, sans le bouger. La coccinelle ouvre une aile, puis part. Elle a volé, là. Tu viens, alors ? Oui, je laisse la rose. Tu as laissé la rose finir. Il a dit oui, après. [pause]</t>
+          <t>J'attends l'&lt;emphasis&gt;envol&lt;/emphasis&gt;. Merci, la rose d'abord. Sarah regarde la rose dans le verre du bocal. La petite bête y marche, à l'envers. Une aile s'ouvre, et l'image s'envole. Elle a volé, là. Tu viens, alors ? Oui, je laisse la rose. Tu as laissé la rose finir. [pause]</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -4372,14 +4372,14 @@
       <c r="AW18" t="inlineStr">
         <is>
           <t>enfant-f|J'attends l'envol.
-copain|Merci, Sarah.
-narrateur|La table garde le bocal, sans le bouger.
-narrateur|La coccinelle ouvre une aile, puis part.
+copain|Merci, la rose d'abord.
+narrateur|Sarah regarde la rose dans le verre du bocal.
+narrateur|La petite bête y marche, à l'envers.
+narrateur|Une aile s'ouvre, et l'image s'envole.
 copain|Elle a volé, là.
 enfant-f|Tu viens, alors ?
 copain|Oui, je laisse la rose.
-papa|Tu as laissé la rose finir.
-maman|Il a dit oui, après.</t>
+papa|Tu as laissé la rose finir.</t>
         </is>
       </c>
       <c r="AX18" t="inlineStr">
@@ -4411,17 +4411,17 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>La rose est vide, à présent. Elle a volé, Sarah. Tu as dit oui, après. Les ailes se sont tues. Le grelot glisse vers la branche. Le bocal garde un toc, tiède contre le bois. Nino souffle sur le verre, minuscule. Il chante, dans le bleu. Une feuille de rose reste collée au verre.</t>
+          <t>La rose est vide, et le verre reflète le ciel. Elle a volé, Sarah. Tu as dit oui, après. Les ailes se sont tues. Le grelot glisse vers la branche. Le bocal garde un toc, tiède contre le bois. Nino souffle sur le verre, minuscule. Il chante, dans le bleu. Une feuille de rose reste collée au verre.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La rose est vide, à présent. Elle a volé, Sarah. Tu as dit oui, après. Les ailes se sont tues. Le grelot glisse vers la branche. Le bocal garde un toc, tiède contre le bois. Nino souffle sur le verre, minuscule. Il chante, dans le bleu. Une feuille de rose reste collée au verre.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La rose est vide, et le verre reflète le ciel. Elle a volé, Sarah. Tu as dit oui, après. Les ailes se sont tues. Le grelot glisse vers la branche. Le bocal garde un toc, tiède contre le bois. Nino souffle sur le verre, minuscule. Il chante, dans le bleu. Une feuille de rose reste collée au verre.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La rose est vide, à présent. Elle a volé, Sarah. Tu as dit oui, après. Les ailes se sont tues. Le grelot glisse vers la branche. Le bocal garde un toc, tiède contre le bois. Nino souffle sur le verre, minuscule. Il chante, dans le bleu. Une feuille de rose reste collée au verre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La rose est vide, et le verre reflète le ciel. Elle a volé, Sarah. Tu as dit oui, après. Les ailes se sont tues. Le grelot glisse vers la branche. Le bocal garde un toc, tiède contre le bois. Nino souffle sur le verre, minuscule. Il chante, dans le bleu. Une feuille de rose reste collée au verre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="AW19" t="inlineStr">
         <is>
-          <t>narrateur|La rose est vide, à présent.
+          <t>narrateur|La rose est vide, et le verre reflète le ciel.
 copain|Elle a volé, Sarah.
 enfant-f|Tu as dit oui, après.
 papa|Les ailes se sont tues.
@@ -4599,17 +4599,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Nino, un grelot minuscule ? Elle fait tinter le verre, près de la rose. Elle l'entend, la petite ? Bas, oui. Une aile se lève, puis se rassoit. On va jusqu'au prunier, alors. D'accord. Le son n'a pas chassé la rose. Il a choisi le voyage.</t>
+          <t>Un toc minuscule, pour elle ? Elle pose le bocal près de la tige, sans frotter. Elle l'entend, la petite ? Bas, oui. Une aile se lève, puis se rassoit sur le col. On va jusqu'au prunier, alors. D'accord. Le son n'a pas chassé la rose. Il a choisi le voyage.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino, un &lt;emphasis level="moderate"&gt;grelot&lt;/emphasis&gt; minuscule ? Elle fait tinter le verre, près de la rose. Elle l'entend, la petite ? Bas, oui. Une aile se lève, puis se rassoit. On va jusqu'au prunier, alors. D'accord. Le son n'a pas chassé la rose. Il a choisi le voyage.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un toc minuscule, pour elle ? Elle pose le bocal près de la tige, sans frotter. Elle l'entend, la petite ? Bas, oui. Une aile se lève, puis se rassoit sur le col. On va jusqu'au prunier, alors. D'accord. Le son n'a pas chassé la rose. Il a choisi le voyage.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Nino, un &lt;emphasis&gt;grelot&lt;/emphasis&gt; minuscule ? Elle fait tinter le verre, près de la rose. Elle l'entend, la petite ? Bas, oui. Une aile se lève, puis se rassoit. On va jusqu'au prunier, alors. D'accord. Le son n'a pas chassé la rose. Il a choisi le voyage. [pause]</t>
+          <t>Un toc minuscule, pour elle ? Elle pose le bocal près de la tige, sans frotter. Elle l'entend, la petite ? Bas, oui. Une aile se lève, puis se rassoit sur le col. On va jusqu'au prunier, alors. D'accord. Le son n'a pas chassé la rose. Il a choisi le voyage. [pause]</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -4743,11 +4743,11 @@
       </c>
       <c r="AW20" t="inlineStr">
         <is>
-          <t>enfant-f|Nino, un grelot minuscule ?
-narrateur|Elle fait tinter le verre, près de la rose.
+          <t>enfant-f|Un toc minuscule, pour elle ?
+narrateur|Elle pose le bocal près de la tige, sans frotter.
 copain|Elle l'entend, la petite ?
 enfant-f|Bas, oui.
-narrateur|Une aile se lève, puis se rassoit.
+narrateur|Une aile se lève, puis se rassoit sur le col.
 copain|On va jusqu'au prunier, alors.
 enfant-f|D'accord.
 papa|Le son n'a pas chassé la rose.
@@ -4971,17 +4971,17 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Pas maintenant, Sarah. D'accord. Elle serre le bocal, les épaules basses. J'accroche ici, alors. Le bocal reste sur la table, à elle. Un toc part vers la rose, loin. Je l'entends, d'ici ! Toi la rose, moi le prunier. Tu as gardé ton carillon. La rose est restée à lui.</t>
+          <t>Pas maintenant, Sarah. D'accord. Elle serre le bocal, les épaules basses. J'accroche à la table, alors. Un toc part vers la rose, loin, sans elle. Je l'entends, d'ici ! Toi la rose, moi le verre. Tu as gardé ton carillon. La rose est restée à lui.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Pas maintenant, Sarah. D'accord. Elle serre le bocal, les épaules basses. J'accroche ici, alors. Le bocal reste sur la table, à elle. Un toc part vers la rose, loin. Je l'entends, d'ici ! Toi la rose, moi le prunier. Tu as gardé ton &lt;emphasis level="moderate"&gt;carillon&lt;/emphasis&gt;. La rose est restée à lui.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Pas maintenant, Sarah. D'accord. Elle serre le bocal, les épaules basses. J'accroche à la table, alors. Un toc part vers la rose, loin, sans elle. Je l'entends, d'ici ! Toi la rose, moi le verre. Tu as gardé ton &lt;emphasis level="moderate"&gt;carillon&lt;/emphasis&gt;. La rose est restée à lui.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Pas maintenant, Sarah. D'accord. Elle serre le bocal, les épaules basses. J'accroche ici, alors. Le bocal reste sur la table, à elle. Un toc part vers la rose, loin. Je l'entends, d'ici ! Toi la rose, moi le prunier. Tu as gardé ton &lt;emphasis&gt;carillon&lt;/emphasis&gt;. La rose est restée à lui. [pause]</t>
+          <t>Pas maintenant, Sarah. D'accord. Elle serre le bocal, les épaules basses. J'accroche à la table, alors. Un toc part vers la rose, loin, sans elle. Je l'entends, d'ici ! Toi la rose, moi le verre. Tu as gardé ton &lt;emphasis&gt;carillon&lt;/emphasis&gt;. La rose est restée à lui. [pause]</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -5118,11 +5118,10 @@
           <t>copain|Pas maintenant, Sarah.
 enfant-f|D'accord.
 narrateur|Elle serre le bocal, les épaules basses.
-enfant-f|J'accroche ici, alors.
-narrateur|Le bocal reste sur la table, à elle.
-narrateur|Un toc part vers la rose, loin.
+enfant-f|J'accroche à la table, alors.
+narrateur|Un toc part vers la rose, loin, sans elle.
 copain|Je l'entends, d'ici !
-enfant-f|Toi la rose, moi le prunier.
+enfant-f|Toi la rose, moi le verre.
 papa|Tu as gardé ton carillon.
 maman|La rose est restée à lui.</t>
         </is>
@@ -5729,17 +5728,17 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>J'aide un peu. Elle fouille sous la table, sans se presser. Une sandale chaude apparaît, collée au pied. Elle s'était cachée ! Près du bord, oui. Deux pieds, à présent, bien chauds. On peut accrocher, là. Tu as cherché avec lui. Le pied nu n'a plus froid.</t>
+          <t>J'aide un peu. Elle penche le bocal, et le verre éclaire l'ombre. Une sandale chaude apparaît, collée au pied de table. Elle s'était cachée sous le bois ! Près du bord, oui. Deux pieds, à présent, bien chauds. On peut accrocher, là. Tu as cherché avec lui. Le pied nu n'a plus froid.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'aide un peu. Elle fouille sous la table, sans se presser. Une &lt;emphasis level="moderate"&gt;sandale&lt;/emphasis&gt; chaude apparaît, collée au pied. Elle s'était cachée ! Près du bord, oui. Deux pieds, à présent, bien chauds. On peut accrocher, là. Tu as cherché avec lui. Le pied nu n'a plus froid.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'aide un peu. Elle penche le bocal, et le verre éclaire l'ombre. Une &lt;emphasis level="moderate"&gt;sandale&lt;/emphasis&gt; chaude apparaît, collée au pied de table. Elle s'était cachée sous le bois ! Près du bord, oui. Deux pieds, à présent, bien chauds. On peut accrocher, là. Tu as cherché avec lui. Le pied nu n'a plus froid.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>J'aide un peu. Elle fouille sous la table, sans se presser. Une &lt;emphasis&gt;sandale&lt;/emphasis&gt; chaude apparaît, collée au pied. Elle s'était cachée ! Près du bord, oui. Deux pieds, à présent, bien chauds. On peut accrocher, là. Tu as cherché avec lui. Le pied nu n'a plus froid. [pause]</t>
+          <t>J'aide un peu. Elle penche le bocal, et le verre éclaire l'ombre. Une &lt;emphasis&gt;sandale&lt;/emphasis&gt; chaude apparaît, collée au pied de table. Elle s'était cachée sous le bois ! Près du bord, oui. Deux pieds, à présent, bien chauds. On peut accrocher, là. Tu as cherché avec lui. Le pied nu n'a plus froid. [pause]</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -5874,9 +5873,9 @@
       <c r="AW26" t="inlineStr">
         <is>
           <t>enfant-f|J'aide un peu.
-narrateur|Elle fouille sous la table, sans se presser.
-narrateur|Une sandale chaude apparaît, collée au pied.
-copain|Elle s'était cachée !
+narrateur|Elle penche le bocal, et le verre éclaire l'ombre.
+narrateur|Une sandale chaude apparaît, collée au pied de table.
+copain|Elle s'était cachée sous le bois !
 enfant-f|Près du bord, oui.
 narrateur|Deux pieds, à présent, bien chauds.
 copain|On peut accrocher, là.
@@ -5913,17 +5912,17 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Les deux sandales sont chaudes, enfin. Le pied nu n'a plus froid. On peut accrocher, là. Vous avez cherché ensemble. La branche attend, un peu. Le bocal garde un toc, tiède contre le bois. Nino s'assoit, le pied au chaud. Le carillon est prêt, pour deux. Les deux sandales fument un peu, au soleil.</t>
+          <t>Les deux sandales fument un peu, sous la table. Le pied nu n'a plus froid. On peut accrocher, là. Vous avez cherché ensemble. La branche attend, un peu. Le bocal garde un toc, tiède contre le bois. Nino s'assoit, le pied au chaud. Le carillon est prêt, pour deux. Les deux sandales fument un peu, au soleil.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les deux sandales sont chaudes, enfin. Le pied nu n'a plus froid. On peut accrocher, là. Vous avez cherché ensemble. La branche attend, un peu. Le bocal garde un toc, tiède contre le bois. Nino s'assoit, le pied au chaud. Le carillon est prêt, pour deux. Les deux sandales fument un peu, au soleil.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les deux sandales fument un peu, sous la table. Le pied nu n'a plus froid. On peut accrocher, là. Vous avez cherché ensemble. La branche attend, un peu. Le bocal garde un toc, tiède contre le bois. Nino s'assoit, le pied au chaud. Le carillon est prêt, pour deux. Les deux sandales fument un peu, au soleil.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les deux sandales sont chaudes, enfin. Le pied nu n'a plus froid. On peut accrocher, là. Vous avez cherché ensemble. La branche attend, un peu. Le bocal garde un toc, tiède contre le bois. Nino s'assoit, le pied au chaud. Le carillon est prêt, pour deux. Les deux sandales fument un peu, au soleil.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les deux sandales fument un peu, sous la table. Le pied nu n'a plus froid. On peut accrocher, là. Vous avez cherché ensemble. La branche attend, un peu. Le bocal garde un toc, tiède contre le bois. Nino s'assoit, le pied au chaud. Le carillon est prêt, pour deux. Les deux sandales fument un peu, au soleil.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -6061,7 +6060,7 @@
       </c>
       <c r="AW27" t="inlineStr">
         <is>
-          <t>narrateur|Les deux sandales sont chaudes, enfin.
+          <t>narrateur|Les deux sandales fument un peu, sous la table.
 copain|Le pied nu n'a plus froid.
 enfant-f|On peut accrocher, là.
 papa|Vous avez cherché ensemble.
@@ -6101,17 +6100,17 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Un petit regard, Nino ? Très petit, alors. D'accord. Ils se penchent vers le bocal, une seconde. Un toc brille, une seconde. Il chante, presque. Puis Nino reprend la sandale. Tu as montré juste un peu. Il a vu, puis choisi.</t>
+          <t>Un petit regard, Nino ? Le temps d'un toc, alors. D'accord. Nino colle l'œil au verre, une seconde. Le jardin y tremble, à l'envers. Il chante, presque. Il lâche le bocal, et reprend la sandale. Tu as montré juste un peu. Il a vu, puis choisi.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un petit &lt;emphasis level="moderate"&gt;regard&lt;/emphasis&gt;, Nino ? Très petit, alors. D'accord. Ils se penchent vers le bocal, une seconde. Un toc brille, une seconde. Il chante, presque. Puis Nino reprend la sandale. Tu as montré juste un peu. Il a vu, puis choisi.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un petit &lt;emphasis level="moderate"&gt;regard&lt;/emphasis&gt;, Nino ? Le temps d'un toc, alors. D'accord. Nino colle l'œil au verre, une seconde. Le jardin y tremble, à l'envers. Il chante, presque. Il lâche le bocal, et reprend la sandale. Tu as montré juste un peu. Il a vu, puis choisi.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Un petit &lt;emphasis&gt;regard&lt;/emphasis&gt;, Nino ? Très petit, alors. D'accord. Ils se penchent vers le bocal, une seconde. Un toc brille, une seconde. Il chante, presque. Puis Nino reprend la sandale. Tu as montré juste un peu. Il a vu, puis choisi. [pause]</t>
+          <t>Un petit &lt;emphasis&gt;regard&lt;/emphasis&gt;, Nino ? Le temps d'un toc, alors. D'accord. Nino colle l'œil au verre, une seconde. Le jardin y tremble, à l'envers. Il chante, presque. Il lâche le bocal, et reprend la sandale. Tu as montré juste un peu. Il a vu, puis choisi. [pause]</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -6246,12 +6245,12 @@
       <c r="AW28" t="inlineStr">
         <is>
           <t>enfant-f|Un petit regard, Nino ?
-copain|Très petit, alors.
+copain|Le temps d'un toc, alors.
 enfant-f|D'accord.
-narrateur|Ils se penchent vers le bocal, une seconde.
-narrateur|Un toc brille, une seconde.
+narrateur|Nino colle l'œil au verre, une seconde.
+narrateur|Le jardin y tremble, à l'envers.
 copain|Il chante, presque.
-narrateur|Puis Nino reprend la sandale.
+narrateur|Il lâche le bocal, et reprend la sandale.
 papa|Tu as montré juste un peu.
 maman|Il a vu, puis choisi.</t>
         </is>
@@ -6473,17 +6472,17 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>On accroche plus tard, alors ? Oui, plus tard. D'accord. La table garde le bocal, pour lui. Nino serre la sandale, concentré. Garde un son pour moi. Il t'attend à la branche. Tu as dit une autre heure. Le pied nu cherche, lui.</t>
+          <t>On accroche plus tard, alors ? Oui, plus tard, le pied d'abord. D'accord. Sarah pose le bocal au milieu de la nappe. Nino serre la sandale, concentré. Garde un toc pour moi. Il t'attend sur le bois. Tu as dit une autre heure. Le pied nu cherche, lui.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On accroche &lt;emphasis level="moderate"&gt;plus tard&lt;/emphasis&gt;, alors ? Oui, plus tard. D'accord. La table garde le bocal, pour lui. Nino serre la sandale, concentré. Garde un son pour moi. Il t'attend à la branche. Tu as dit une autre heure. Le pied nu cherche, lui.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On accroche &lt;emphasis level="moderate"&gt;plus tard&lt;/emphasis&gt;, alors ? Oui, plus tard, le pied d'abord. D'accord. Sarah pose le bocal au milieu de la nappe. Nino serre la sandale, concentré. Garde un toc pour moi. Il t'attend sur le bois. Tu as dit une autre heure. Le pied nu cherche, lui.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>On accroche &lt;emphasis&gt;plus tard&lt;/emphasis&gt;, alors ? Oui, plus tard. D'accord. La table garde le bocal, pour lui. Nino serre la sandale, concentré. Garde un son pour moi. Il t'attend à la branche. Tu as dit une autre heure. Le pied nu cherche, lui. [pause]</t>
+          <t>On accroche &lt;emphasis&gt;plus tard&lt;/emphasis&gt;, alors ? Oui, plus tard, le pied d'abord. D'accord. Sarah pose le bocal au milieu de la nappe. Nino serre la sandale, concentré. Garde un toc pour moi. Il t'attend sur le bois. Tu as dit une autre heure. Le pied nu cherche, lui. [pause]</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -6618,12 +6617,12 @@
       <c r="AW30" t="inlineStr">
         <is>
           <t>enfant-f|On accroche plus tard, alors ?
-copain|Oui, plus tard.
+copain|Oui, plus tard, le pied d'abord.
 enfant-f|D'accord.
-narrateur|La table garde le bocal, pour lui.
+narrateur|Sarah pose le bocal au milieu de la nappe.
 narrateur|Nino serre la sandale, concentré.
-copain|Garde un son pour moi.
-enfant-f|Il t'attend à la branche.
+copain|Garde un toc pour moi.
+enfant-f|Il t'attend sur le bois.
 papa|Tu as dit une autre heure.
 maman|Le pied nu cherche, lui.</t>
         </is>
@@ -7983,17 +7982,17 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>J'attends le dernier trait. Merci, Sarah. Elle compte les rayons sur le fer froid. Le grelot attend sur la marche, silencieux. La craie s'arrête, pile. Il a son soleil, là. Tu viens, alors ? Oui, j'apporte la craie. Tu as laissé le soleil finir.</t>
+          <t>J'attends le dernier trait. Merci, le grelot après le trait. Sarah tient le fer, le doigt sur la languette. Le grelot reste muet, sur la marche froide. Nino tire le rayon, sans un tintement. Il est fini, et ton fer n'a pas volé. Tu viens, alors ? Oui, j'apporte la craie. Tu as gardé le son pour la fin.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'attends le dernier trait. Merci, Sarah. Elle compte les rayons sur le fer froid. Le grelot attend sur la marche, silencieux. La craie s'arrête, pile. Il a son &lt;emphasis level="moderate"&gt;soleil&lt;/emphasis&gt;, là. Tu viens, alors ? Oui, j'apporte la craie. Tu as laissé le soleil finir.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'attends le dernier trait. Merci, le grelot après le trait. Sarah tient le fer, le doigt sur la languette. Le grelot reste muet, sur la marche froide. Nino tire le rayon, sans un tintement. Il est fini, et ton fer n'a pas volé. Tu viens, alors ? Oui, j'apporte la craie. Tu as gardé le son pour la fin.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>J'attends le dernier trait. Merci, Sarah. Elle compte les rayons sur le fer froid. Le grelot attend sur la marche, silencieux. La craie s'arrête, pile. Il a son &lt;emphasis&gt;soleil&lt;/emphasis&gt;, là. Tu viens, alors ? Oui, j'apporte la craie. Tu as laissé le soleil finir. [pause]</t>
+          <t>J'attends le dernier trait. Merci, le grelot après le trait. Sarah tient le fer, le doigt sur la languette. Le grelot reste muet, sur la marche froide. Nino tire le rayon, sans un tintement. Il est fini, et ton fer n'a pas volé. Tu viens, alors ? Oui, j'apporte la craie. Tu as gardé le son pour la fin. [pause]</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
@@ -8128,14 +8127,14 @@
       <c r="AW38" t="inlineStr">
         <is>
           <t>enfant-f|J'attends le dernier trait.
-copain|Merci, Sarah.
-narrateur|Elle compte les rayons sur le fer froid.
-narrateur|Le grelot attend sur la marche, silencieux.
-narrateur|La craie s'arrête, pile.
-copain|Il a son soleil, là.
+copain|Merci, le grelot après le trait.
+narrateur|Sarah tient le fer, le doigt sur la languette.
+narrateur|Le grelot reste muet, sur la marche froide.
+narrateur|Nino tire le rayon, sans un tintement.
+copain|Il est fini, et ton fer n'a pas volé.
 enfant-f|Tu viens, alors ?
 copain|Oui, j'apporte la craie.
-papa|Tu as laissé le soleil finir.</t>
+papa|Tu as gardé le son pour la fin.</t>
         </is>
       </c>
       <c r="AX38" t="inlineStr">
@@ -8167,17 +8166,17 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Le soleil de craie reste sur la pierre. Il a son dernier trait, Sarah. Oui, tout jaune. La craie a laissé la place. Le prunier fait un petit toc. Le grelot dort contre le verre, minuscule. Nino noue le ruban, les doigts tâchés de jaune. Le jardin chante, là. Le grelot et le soleil de craie se touchent.</t>
+          <t>Le soleil de craie borde la marche de pierre. Il a son dernier trait, Sarah. Oui, bien jaune. La craie a laissé la place. Le prunier fait un petit toc. Le grelot dort contre le verre, minuscule. Nino noue le ruban, les doigts tâchés de jaune. Le jardin chante, là. Le grelot et le soleil de craie se touchent.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le soleil de craie reste sur la pierre. Il a son dernier trait, Sarah. Oui, tout jaune. La craie a laissé la place. Le &lt;emphasis level="moderate"&gt;prunier&lt;/emphasis&gt; fait un petit toc. Le grelot dort contre le verre, minuscule. Nino noue le ruban, les doigts tâchés de jaune. Le jardin chante, là. Le grelot et le soleil de craie se touchent.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le soleil de craie borde la marche de pierre. Il a son dernier trait, Sarah. Oui, bien jaune. La craie a laissé la place. Le &lt;emphasis level="moderate"&gt;prunier&lt;/emphasis&gt; fait un petit toc. Le grelot dort contre le verre, minuscule. Nino noue le ruban, les doigts tâchés de jaune. Le jardin chante, là. Le grelot et le soleil de craie se touchent.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le soleil de craie reste sur la pierre. Il a son dernier trait, Sarah. Oui, tout jaune. La craie a laissé la place. Le &lt;emphasis&gt;prunier&lt;/emphasis&gt; fait un petit toc. Le grelot dort contre le verre, minuscule. Nino noue le ruban, les doigts tâchés de jaune. Le jardin chante, là. Le grelot et le soleil de craie se touchent.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le soleil de craie borde la marche de pierre. Il a son dernier trait, Sarah. Oui, bien jaune. La craie a laissé la place. Le &lt;emphasis&gt;prunier&lt;/emphasis&gt; fait un petit toc. Le grelot dort contre le verre, minuscule. Nino noue le ruban, les doigts tâchés de jaune. Le jardin chante, là. Le grelot et le soleil de craie se touchent.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
@@ -8315,9 +8314,9 @@
       </c>
       <c r="AW39" t="inlineStr">
         <is>
-          <t>narrateur|Le soleil de craie reste sur la pierre.
+          <t>narrateur|Le soleil de craie borde la marche de pierre.
 copain|Il a son dernier trait, Sarah.
-enfant-f|Oui, tout jaune.
+enfant-f|Oui, bien jaune.
 papa|La craie a laissé la place.
 maman|Le prunier fait un petit toc.
 narrateur|Le grelot dort contre le verre, minuscule.
@@ -8355,17 +8354,17 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Nino, un carillon t'écoute. Elle glisse le grelot contre le soleil. Sa voix reste près de lui, presque un souffle. Il a une oreille, lui aussi ? Oui, minuscule comme un rayon. Je viens, alors. Il pose la craie, sans la perdre. Tu as parlé contre son dessin. C'est lui qui a dit oui.</t>
+          <t>Nino, un tintement pour le rayon ? Elle ouvre le poing, juste au-dessus du jaune. Un son mince montre le trait qui manque. Il m'a montré où tirer. Minuscule, comme un rayon. Je viens, alors. Il pose la craie contre le petit fer. Le son a aidé le dessin, pas volé. C'est lui qui a dit oui.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino, un &lt;emphasis level="moderate"&gt;carillon&lt;/emphasis&gt; t'écoute. Elle glisse le grelot contre le soleil. Sa voix reste près de lui, presque un souffle. Il a une oreille, lui aussi ? Oui, minuscule comme un rayon. Je viens, alors. Il pose la craie, sans la perdre. Tu as parlé contre son dessin. C'est lui qui a dit oui.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino, un tintement pour le rayon ? Elle ouvre le poing, juste au-dessus du jaune. Un son mince montre le trait qui manque. Il m'a montré où tirer. Minuscule, comme un rayon. Je viens, alors. Il pose la craie contre le petit fer. Le son a aidé le dessin, pas volé. C'est lui qui a dit oui.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Nino, un &lt;emphasis&gt;carillon&lt;/emphasis&gt; t'écoute. Elle glisse le grelot contre le soleil. Sa voix reste près de lui, presque un souffle. Il a une oreille, lui aussi ? Oui, minuscule comme un rayon. Je viens, alors. Il pose la craie, sans la perdre. Tu as parlé contre son dessin. C'est lui qui a dit oui. [pause]</t>
+          <t>Nino, un tintement pour le rayon ? Elle ouvre le poing, juste au-dessus du jaune. Un son mince montre le trait qui manque. Il m'a montré où tirer. Minuscule, comme un rayon. Je viens, alors. Il pose la craie contre le petit fer. Le son a aidé le dessin, pas volé. C'est lui qui a dit oui. [pause]</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
@@ -8499,14 +8498,14 @@
       </c>
       <c r="AW40" t="inlineStr">
         <is>
-          <t>enfant-f|Nino, un carillon t'écoute.
-narrateur|Elle glisse le grelot contre le soleil.
-narrateur|Sa voix reste près de lui, presque un souffle.
-copain|Il a une oreille, lui aussi ?
-enfant-f|Oui, minuscule comme un rayon.
+          <t>enfant-f|Nino, un tintement pour le rayon ?
+narrateur|Elle ouvre le poing, juste au-dessus du jaune.
+narrateur|Un son mince montre le trait qui manque.
+copain|Il m'a montré où tirer.
+enfant-f|Minuscule, comme un rayon.
 copain|Je viens, alors.
-narrateur|Il pose la craie, sans la perdre.
-papa|Tu as parlé contre son dessin.
+narrateur|Il pose la craie contre le petit fer.
+papa|Le son a aidé le dessin, pas volé.
 maman|C'est lui qui a dit oui.</t>
         </is>
       </c>
@@ -8727,17 +8726,17 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Je m'assois à côté. Sarah s'assoit sur la marche de pierre. Elle ne touche pas la craie. Tu vois le rayon, toi aussi ? Oui, il pique un peu. Un dernier trait les fait souffler. On accroche, après ça. Tu as écouté son soleil. C'est lui qui a dit après.</t>
+          <t>Je m'assois à côté. Sarah s'assoit sur la marche de pierre. Le grelot dort sur ses genoux, silencieux. Ta cloche a chaud, là ? Oui, elle attend ton trait. Un dernier trait les fait souffler ensemble. On accroche, après ça. Tu as écouté son soleil. C'est lui qui a dit après.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Je m'assois à &lt;emphasis level="moderate"&gt;côté&lt;/emphasis&gt;. Sarah s'assoit sur la marche de pierre. Elle ne touche pas la craie. Tu vois le rayon, toi aussi ? Oui, il pique un peu. Un dernier trait les fait souffler. On accroche, après ça. Tu as écouté son soleil. C'est lui qui a dit après.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Je m'assois à &lt;emphasis level="moderate"&gt;côté&lt;/emphasis&gt;. Sarah s'assoit sur la marche de pierre. Le grelot dort sur ses genoux, silencieux. Ta cloche a chaud, là ? Oui, elle attend ton trait. Un dernier trait les fait souffler ensemble. On accroche, après ça. Tu as écouté son soleil. C'est lui qui a dit après.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Je m'assois à &lt;emphasis&gt;côté&lt;/emphasis&gt;. Sarah s'assoit sur la marche de pierre. Elle ne touche pas la craie. Tu vois le rayon, toi aussi ? Oui, il pique un peu. Un dernier trait les fait souffler. On accroche, après ça. Tu as écouté son soleil. C'est lui qui a dit après. [pause]</t>
+          <t>Je m'assois à &lt;emphasis&gt;côté&lt;/emphasis&gt;. Sarah s'assoit sur la marche de pierre. Le grelot dort sur ses genoux, silencieux. Ta cloche a chaud, là ? Oui, elle attend ton trait. Un dernier trait les fait souffler ensemble. On accroche, après ça. Tu as écouté son soleil. C'est lui qui a dit après. [pause]</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -8873,10 +8872,10 @@
         <is>
           <t>enfant-f|Je m'assois à côté.
 narrateur|Sarah s'assoit sur la marche de pierre.
-narrateur|Elle ne touche pas la craie.
-copain|Tu vois le rayon, toi aussi ?
-enfant-f|Oui, il pique un peu.
-narrateur|Un dernier trait les fait souffler.
+narrateur|Le grelot dort sur ses genoux, silencieux.
+copain|Ta cloche a chaud, là ?
+enfant-f|Oui, elle attend ton trait.
+narrateur|Un dernier trait les fait souffler ensemble.
 copain|On accroche, après ça.
 papa|Tu as écouté son soleil.
 maman|C'est lui qui a dit après.</t>
@@ -9484,17 +9483,17 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>J'attends l'envol. Merci, Sarah. Le grelot dort dans sa paume, sans son. La coccinelle ouvre une aile, puis part. Elle a volé, là. Tu viens, alors ? Oui, je laisse la rose. Tu as laissé la rose finir. Il a dit oui, après.</t>
+          <t>J'attends l'envol. Merci, pas de son. Sarah ferme le poing, le grelot prisonnier. La rose n'entend que le souffle de Nino. Une aile s'ouvre, et la petite part. Elle a volé, sans peur. Tu viens, alors ? Oui, je laisse la rose. Tu as laissé la rose finir.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'attends l'&lt;emphasis level="moderate"&gt;envol&lt;/emphasis&gt;. Merci, Sarah. Le grelot dort dans sa paume, sans son. La coccinelle ouvre une aile, puis part. Elle a volé, là. Tu viens, alors ? Oui, je laisse la rose. Tu as laissé la rose finir. Il a dit oui, après.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'attends l'&lt;emphasis level="moderate"&gt;envol&lt;/emphasis&gt;. Merci, pas de son. Sarah ferme le poing, le grelot prisonnier. La rose n'entend que le souffle de Nino. Une aile s'ouvre, et la petite part. Elle a volé, sans peur. Tu viens, alors ? Oui, je laisse la rose. Tu as laissé la rose finir.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>J'attends l'&lt;emphasis&gt;envol&lt;/emphasis&gt;. Merci, Sarah. Le grelot dort dans sa paume, sans son. La coccinelle ouvre une aile, puis part. Elle a volé, là. Tu viens, alors ? Oui, je laisse la rose. Tu as laissé la rose finir. Il a dit oui, après. [pause]</t>
+          <t>J'attends l'&lt;emphasis&gt;envol&lt;/emphasis&gt;. Merci, pas de son. Sarah ferme le poing, le grelot prisonnier. La rose n'entend que le souffle de Nino. Une aile s'ouvre, et la petite part. Elle a volé, sans peur. Tu viens, alors ? Oui, je laisse la rose. Tu as laissé la rose finir. [pause]</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -9629,14 +9628,14 @@
       <c r="AW46" t="inlineStr">
         <is>
           <t>enfant-f|J'attends l'envol.
-copain|Merci, Sarah.
-narrateur|Le grelot dort dans sa paume, sans son.
-narrateur|La coccinelle ouvre une aile, puis part.
-copain|Elle a volé, là.
+copain|Merci, pas de son.
+narrateur|Sarah ferme le poing, le grelot prisonnier.
+narrateur|La rose n'entend que le souffle de Nino.
+narrateur|Une aile s'ouvre, et la petite part.
+copain|Elle a volé, sans peur.
 enfant-f|Tu viens, alors ?
 copain|Oui, je laisse la rose.
-papa|Tu as laissé la rose finir.
-maman|Il a dit oui, après.</t>
+papa|Tu as laissé la rose finir.</t>
         </is>
       </c>
       <c r="AX46" t="inlineStr">
@@ -9668,17 +9667,17 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>La rose est vide, à présent. Elle a volé, Sarah. Tu as dit oui, après. Les ailes se sont tues. Le grelot glisse vers la branche. Le grelot dort contre le verre, minuscule. Nino souffle sur le fer, minuscule. Il chante, dans le bleu. La rose vide sent le chaud du soir.</t>
+          <t>La rose est vide, et le fer reste froid. Elle a volé, Sarah. Tu as dit oui, après. Les ailes se sont tues. Le grelot glisse vers la branche. Le grelot dort contre le verre, minuscule. Nino souffle sur le fer, minuscule. Il chante, dans le bleu. La rose vide sent le chaud du soir.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La rose est vide, à présent. Elle a volé, Sarah. Tu as dit oui, après. Les ailes se sont tues. Le grelot glisse vers la branche. Le grelot dort contre le verre, minuscule. Nino souffle sur le fer, minuscule. Il chante, dans le bleu. La rose vide sent le chaud du soir.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La rose est vide, et le fer reste froid. Elle a volé, Sarah. Tu as dit oui, après. Les ailes se sont tues. Le grelot glisse vers la branche. Le grelot dort contre le verre, minuscule. Nino souffle sur le fer, minuscule. Il chante, dans le bleu. La rose vide sent le chaud du soir.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La rose est vide, à présent. Elle a volé, Sarah. Tu as dit oui, après. Les ailes se sont tues. Le grelot glisse vers la branche. Le grelot dort contre le verre, minuscule. Nino souffle sur le fer, minuscule. Il chante, dans le bleu. La rose vide sent le chaud du soir.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La rose est vide, et le fer reste froid. Elle a volé, Sarah. Tu as dit oui, après. Les ailes se sont tues. Le grelot glisse vers la branche. Le grelot dort contre le verre, minuscule. Nino souffle sur le fer, minuscule. Il chante, dans le bleu. La rose vide sent le chaud du soir.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -9816,7 +9815,7 @@
       </c>
       <c r="AW47" t="inlineStr">
         <is>
-          <t>narrateur|La rose est vide, à présent.
+          <t>narrateur|La rose est vide, et le fer reste froid.
 copain|Elle a volé, Sarah.
 enfant-f|Tu as dit oui, après.
 papa|Les ailes se sont tues.
@@ -9856,17 +9855,17 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Nino, un grelot minuscule ? Elle ouvre le poing, un son tout mince. Elle l'entend, la petite ? Bas, oui. Une aile se lève, puis se rassoit. On va jusqu'au prunier, alors. D'accord. Le son n'a pas chassé la rose. Il a choisi le voyage.</t>
+          <t>Nino, un grelot minuscule ? Elle ouvre le poing, un son mince comme un fil. Elle l'entend, la petite ? Bas, oui. Une aile se lève, puis se rassoit sur le fer. On va jusqu'au prunier, alors. D'accord. Le son n'a pas chassé la rose. Il a choisi le voyage.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino, un &lt;emphasis level="moderate"&gt;grelot&lt;/emphasis&gt; minuscule ? Elle ouvre le poing, un son tout mince. Elle l'entend, la petite ? Bas, oui. Une aile se lève, puis se rassoit. On va jusqu'au prunier, alors. D'accord. Le son n'a pas chassé la rose. Il a choisi le voyage.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino, un &lt;emphasis level="moderate"&gt;grelot&lt;/emphasis&gt; minuscule ? Elle ouvre le poing, un son mince comme un fil. Elle l'entend, la petite ? Bas, oui. Une aile se lève, puis se rassoit sur le fer. On va jusqu'au prunier, alors. D'accord. Le son n'a pas chassé la rose. Il a choisi le voyage.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Nino, un &lt;emphasis&gt;grelot&lt;/emphasis&gt; minuscule ? Elle ouvre le poing, un son tout mince. Elle l'entend, la petite ? Bas, oui. Une aile se lève, puis se rassoit. On va jusqu'au prunier, alors. D'accord. Le son n'a pas chassé la rose. Il a choisi le voyage. [pause]</t>
+          <t>Nino, un &lt;emphasis&gt;grelot&lt;/emphasis&gt; minuscule ? Elle ouvre le poing, un son mince comme un fil. Elle l'entend, la petite ? Bas, oui. Une aile se lève, puis se rassoit sur le fer. On va jusqu'au prunier, alors. D'accord. Le son n'a pas chassé la rose. Il a choisi le voyage. [pause]</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -10001,10 +10000,10 @@
       <c r="AW48" t="inlineStr">
         <is>
           <t>enfant-f|Nino, un grelot minuscule ?
-narrateur|Elle ouvre le poing, un son tout mince.
+narrateur|Elle ouvre le poing, un son mince comme un fil.
 copain|Elle l'entend, la petite ?
 enfant-f|Bas, oui.
-narrateur|Une aile se lève, puis se rassoit.
+narrateur|Une aile se lève, puis se rassoit sur le fer.
 copain|On va jusqu'au prunier, alors.
 enfant-f|D'accord.
 papa|Le son n'a pas chassé la rose.
@@ -10228,17 +10227,17 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Pas maintenant, Sarah. D'accord. Elle serre le grelot, les épaules basses. J'accroche ici, alors. Le grelot reste dans sa paume, à elle. Un tintement part vers la rose, loin. Je l'entends, d'ici ! Toi la rose, moi le prunier. Tu as gardé ton carillon. La rose est restée à lui.</t>
+          <t>Pas maintenant, Sarah. D'accord. Elle serre le grelot, les épaules basses. J'accroche à la marche, alors. Un tintement part vers la rose, loin. Je l'entends, d'ici ! Toi la rose, moi la pierre. Tu as gardé ton carillon. La rose est restée à lui.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Pas maintenant, Sarah. D'accord. Elle serre le grelot, les épaules basses. J'accroche ici, alors. Le grelot reste dans sa paume, à elle. Un tintement part vers la rose, loin. Je l'entends, d'ici ! Toi la rose, moi le prunier. Tu as gardé ton &lt;emphasis level="moderate"&gt;carillon&lt;/emphasis&gt;. La rose est restée à lui.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Pas maintenant, Sarah. D'accord. Elle serre le grelot, les épaules basses. J'accroche à la marche, alors. Un tintement part vers la rose, loin. Je l'entends, d'ici ! Toi la rose, moi la pierre. Tu as gardé ton &lt;emphasis level="moderate"&gt;carillon&lt;/emphasis&gt;. La rose est restée à lui.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Pas maintenant, Sarah. D'accord. Elle serre le grelot, les épaules basses. J'accroche ici, alors. Le grelot reste dans sa paume, à elle. Un tintement part vers la rose, loin. Je l'entends, d'ici ! Toi la rose, moi le prunier. Tu as gardé ton &lt;emphasis&gt;carillon&lt;/emphasis&gt;. La rose est restée à lui. [pause]</t>
+          <t>Pas maintenant, Sarah. D'accord. Elle serre le grelot, les épaules basses. J'accroche à la marche, alors. Un tintement part vers la rose, loin. Je l'entends, d'ici ! Toi la rose, moi la pierre. Tu as gardé ton &lt;emphasis&gt;carillon&lt;/emphasis&gt;. La rose est restée à lui. [pause]</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -10375,11 +10374,10 @@
           <t>copain|Pas maintenant, Sarah.
 enfant-f|D'accord.
 narrateur|Elle serre le grelot, les épaules basses.
-enfant-f|J'accroche ici, alors.
-narrateur|Le grelot reste dans sa paume, à elle.
+enfant-f|J'accroche à la marche, alors.
 narrateur|Un tintement part vers la rose, loin.
 copain|Je l'entends, d'ici !
-enfant-f|Toi la rose, moi le prunier.
+enfant-f|Toi la rose, moi la pierre.
 papa|Tu as gardé ton carillon.
 maman|La rose est restée à lui.</t>
         </is>
@@ -10986,17 +10984,17 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>J'aide un peu. Elle fouille près de la marche, sans se presser. Une sandale chaude apparaît, collée à la pierre. Elle s'était cachée ! Près du bord, oui. Deux pieds, à présent, bien chauds. On peut accrocher, là. Tu as cherché avec lui. Le pied nu n'a plus froid.</t>
+          <t>J'aide un peu. Elle fait tinter le grelot, près de l'herbe. Le son montre une lanière, collée à la pierre. Elle s'était cachée sous la marche ! Près du bord, oui. Deux pieds, à présent, bien chauds. On peut accrocher, là. Tu as cherché avec lui. Le pied nu n'a plus froid.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'aide un peu. Elle fouille près de la marche, sans se presser. Une &lt;emphasis level="moderate"&gt;sandale&lt;/emphasis&gt; chaude apparaît, collée à la pierre. Elle s'était cachée ! Près du bord, oui. Deux pieds, à présent, bien chauds. On peut accrocher, là. Tu as cherché avec lui. Le pied nu n'a plus froid.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'aide un peu. Elle fait tinter le grelot, près de l'herbe. Le son montre une lanière, collée à la pierre. Elle s'était cachée sous la marche ! Près du bord, oui. Deux pieds, à présent, bien chauds. On peut accrocher, là. Tu as cherché avec lui. Le pied nu n'a plus froid.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>J'aide un peu. Elle fouille près de la marche, sans se presser. Une &lt;emphasis&gt;sandale&lt;/emphasis&gt; chaude apparaît, collée à la pierre. Elle s'était cachée ! Près du bord, oui. Deux pieds, à présent, bien chauds. On peut accrocher, là. Tu as cherché avec lui. Le pied nu n'a plus froid. [pause]</t>
+          <t>J'aide un peu. Elle fait tinter le grelot, près de l'herbe. Le son montre une lanière, collée à la pierre. Elle s'était cachée sous la marche ! Près du bord, oui. Deux pieds, à présent, bien chauds. On peut accrocher, là. Tu as cherché avec lui. Le pied nu n'a plus froid. [pause]</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -11131,9 +11129,9 @@
       <c r="AW54" t="inlineStr">
         <is>
           <t>enfant-f|J'aide un peu.
-narrateur|Elle fouille près de la marche, sans se presser.
-narrateur|Une sandale chaude apparaît, collée à la pierre.
-copain|Elle s'était cachée !
+narrateur|Elle fait tinter le grelot, près de l'herbe.
+narrateur|Le son montre une lanière, collée à la pierre.
+copain|Elle s'était cachée sous la marche !
 enfant-f|Près du bord, oui.
 narrateur|Deux pieds, à présent, bien chauds.
 copain|On peut accrocher, là.
@@ -11170,17 +11168,17 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Les deux sandales sont chaudes, enfin. Le pied nu n'a plus froid. On peut accrocher, là. Vous avez cherché ensemble. La branche attend, un peu. Le grelot dort contre le verre, minuscule. Nino s'assoit, le pied au chaud. Le carillon est prêt, pour deux. Le grelot a montré l'herbe, puis la branche.</t>
+          <t>Les deux sandales fument un peu, près de la marche. Le pied nu n'a plus froid. On peut accrocher, là. Vous avez cherché ensemble. La branche attend, un peu. Le grelot dort contre le verre, minuscule. Nino s'assoit, le pied au chaud. Le carillon est prêt, pour deux. Le grelot a montré l'herbe, puis la branche.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les deux sandales sont chaudes, enfin. Le pied nu n'a plus froid. On peut accrocher, là. Vous avez cherché ensemble. La branche attend, un peu. Le grelot dort contre le verre, minuscule. Nino s'assoit, le pied au chaud. Le carillon est prêt, pour deux. Le grelot a montré l'herbe, puis la branche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les deux sandales fument un peu, près de la marche. Le pied nu n'a plus froid. On peut accrocher, là. Vous avez cherché ensemble. La branche attend, un peu. Le grelot dort contre le verre, minuscule. Nino s'assoit, le pied au chaud. Le carillon est prêt, pour deux. Le grelot a montré l'herbe, puis la branche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les deux sandales sont chaudes, enfin. Le pied nu n'a plus froid. On peut accrocher, là. Vous avez cherché ensemble. La branche attend, un peu. Le grelot dort contre le verre, minuscule. Nino s'assoit, le pied au chaud. Le carillon est prêt, pour deux. Le grelot a montré l'herbe, puis la branche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les deux sandales fument un peu, près de la marche. Le pied nu n'a plus froid. On peut accrocher, là. Vous avez cherché ensemble. La branche attend, un peu. Le grelot dort contre le verre, minuscule. Nino s'assoit, le pied au chaud. Le carillon est prêt, pour deux. Le grelot a montré l'herbe, puis la branche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -11318,7 +11316,7 @@
       </c>
       <c r="AW55" t="inlineStr">
         <is>
-          <t>narrateur|Les deux sandales sont chaudes, enfin.
+          <t>narrateur|Les deux sandales fument un peu, près de la marche.
 copain|Le pied nu n'a plus froid.
 enfant-f|On peut accrocher, là.
 papa|Vous avez cherché ensemble.
@@ -11358,17 +11356,17 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Un petit regard, Nino ? Très petit, alors. D'accord. Ils se penchent vers le grelot, une seconde. Un tintement brille, une seconde. Il chante, presque. Puis Nino reprend la sandale. Tu as montré juste un peu. Il a vu, puis choisi.</t>
+          <t>Un petit regard, Nino ? Le temps d'un tintement, alors. D'accord. Sarah pose le grelot dans sa paume ouverte. Nino le touche du doigt, et le fer dit toc. Assez, je l'ai entendu. Il referme la main de Sarah, puis cherche. Tu as montré juste un peu. Il a vu, puis choisi.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un petit &lt;emphasis level="moderate"&gt;regard&lt;/emphasis&gt;, Nino ? Très petit, alors. D'accord. Ils se penchent vers le grelot, une seconde. Un tintement brille, une seconde. Il chante, presque. Puis Nino reprend la sandale. Tu as montré juste un peu. Il a vu, puis choisi.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un petit &lt;emphasis level="moderate"&gt;regard&lt;/emphasis&gt;, Nino ? Le temps d'un tintement, alors. D'accord. Sarah pose le grelot dans sa paume ouverte. Nino le touche du doigt, et le fer dit toc. Assez, je l'ai entendu. Il referme la main de Sarah, puis cherche. Tu as montré juste un peu. Il a vu, puis choisi.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Un petit &lt;emphasis&gt;regard&lt;/emphasis&gt;, Nino ? Très petit, alors. D'accord. Ils se penchent vers le grelot, une seconde. Un tintement brille, une seconde. Il chante, presque. Puis Nino reprend la sandale. Tu as montré juste un peu. Il a vu, puis choisi. [pause]</t>
+          <t>Un petit &lt;emphasis&gt;regard&lt;/emphasis&gt;, Nino ? Le temps d'un tintement, alors. D'accord. Sarah pose le grelot dans sa paume ouverte. Nino le touche du doigt, et le fer dit toc. Assez, je l'ai entendu. Il referme la main de Sarah, puis cherche. Tu as montré juste un peu. Il a vu, puis choisi. [pause]</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -11503,12 +11501,12 @@
       <c r="AW56" t="inlineStr">
         <is>
           <t>enfant-f|Un petit regard, Nino ?
-copain|Très petit, alors.
+copain|Le temps d'un tintement, alors.
 enfant-f|D'accord.
-narrateur|Ils se penchent vers le grelot, une seconde.
-narrateur|Un tintement brille, une seconde.
-copain|Il chante, presque.
-narrateur|Puis Nino reprend la sandale.
+narrateur|Sarah pose le grelot dans sa paume ouverte.
+narrateur|Nino le touche du doigt, et le fer dit toc.
+copain|Assez, je l'ai entendu.
+narrateur|Il referme la main de Sarah, puis cherche.
 papa|Tu as montré juste un peu.
 maman|Il a vu, puis choisi.</t>
         </is>
@@ -11730,17 +11728,17 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>On accroche plus tard, alors ? Oui, plus tard. D'accord. La marche garde le grelot, pour lui. Nino serre la sandale, concentré. Garde un son pour moi. Il t'attend à la branche. Tu as dit une autre heure. Le pied nu cherche, lui.</t>
+          <t>On accroche plus tard, alors ? Oui, plus tard, le pied d'abord. D'accord. Sarah pose le grelot au bord de la marche. Nino serre la sandale, concentré. Garde un tintement pour moi. Il t'attend sur la pierre. Tu as dit une autre heure. Le pied nu cherche, lui.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On accroche &lt;emphasis level="moderate"&gt;plus tard&lt;/emphasis&gt;, alors ? Oui, plus tard. D'accord. La marche garde le grelot, pour lui. Nino serre la sandale, concentré. Garde un son pour moi. Il t'attend à la branche. Tu as dit une autre heure. Le pied nu cherche, lui.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On accroche &lt;emphasis level="moderate"&gt;plus tard&lt;/emphasis&gt;, alors ? Oui, plus tard, le pied d'abord. D'accord. Sarah pose le grelot au bord de la marche. Nino serre la sandale, concentré. Garde un tintement pour moi. Il t'attend sur la pierre. Tu as dit une autre heure. Le pied nu cherche, lui.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>On accroche &lt;emphasis&gt;plus tard&lt;/emphasis&gt;, alors ? Oui, plus tard. D'accord. La marche garde le grelot, pour lui. Nino serre la sandale, concentré. Garde un son pour moi. Il t'attend à la branche. Tu as dit une autre heure. Le pied nu cherche, lui. [pause]</t>
+          <t>On accroche &lt;emphasis&gt;plus tard&lt;/emphasis&gt;, alors ? Oui, plus tard, le pied d'abord. D'accord. Sarah pose le grelot au bord de la marche. Nino serre la sandale, concentré. Garde un tintement pour moi. Il t'attend sur la pierre. Tu as dit une autre heure. Le pied nu cherche, lui. [pause]</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -11875,12 +11873,12 @@
       <c r="AW58" t="inlineStr">
         <is>
           <t>enfant-f|On accroche plus tard, alors ?
-copain|Oui, plus tard.
+copain|Oui, plus tard, le pied d'abord.
 enfant-f|D'accord.
-narrateur|La marche garde le grelot, pour lui.
+narrateur|Sarah pose le grelot au bord de la marche.
 narrateur|Nino serre la sandale, concentré.
-copain|Garde un son pour moi.
-enfant-f|Il t'attend à la branche.
+copain|Garde un tintement pour moi.
+enfant-f|Il t'attend sur la pierre.
 papa|Tu as dit une autre heure.
 maman|Le pied nu cherche, lui.</t>
         </is>
@@ -13239,17 +13237,17 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>J'attends le dernier trait. Merci, Sarah. Elle compte les rayons sur le ruban bleu. Le ruban attend à la branche, vide. La craie s'arrête, pile. Il a son soleil, là. Tu viens, alors ? Oui, j'apporte la craie. Tu as laissé le soleil finir.</t>
+          <t>J'attends le dernier trait. Merci, ta boucle après. Sarah enroule le ruban autour d'un doigt. Chaque tour compte un rayon, sans tirer Nino. La craie s'arrête, et le bleu se desserre. Mon soleil est rond, comme ta boucle. Tu viens, alors ? Oui, j'apporte la craie. Tu as laissé le soleil finir.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'attends le dernier trait. Merci, Sarah. Elle compte les rayons sur le ruban bleu. Le ruban attend à la branche, vide. La craie s'arrête, pile. Il a son &lt;emphasis level="moderate"&gt;soleil&lt;/emphasis&gt;, là. Tu viens, alors ? Oui, j'apporte la craie. Tu as laissé le soleil finir.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'attends le dernier trait. Merci, ta boucle après. Sarah enroule le ruban autour d'un doigt. Chaque tour compte un rayon, sans tirer Nino. La craie s'arrête, et le bleu se desserre. Mon &lt;emphasis level="moderate"&gt;soleil&lt;/emphasis&gt; est rond, comme ta boucle. Tu viens, alors ? Oui, j'apporte la craie. Tu as laissé le soleil finir.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>J'attends le dernier trait. Merci, Sarah. Elle compte les rayons sur le ruban bleu. Le ruban attend à la branche, vide. La craie s'arrête, pile. Il a son &lt;emphasis&gt;soleil&lt;/emphasis&gt;, là. Tu viens, alors ? Oui, j'apporte la craie. Tu as laissé le soleil finir. [pause]</t>
+          <t>J'attends le dernier trait. Merci, ta boucle après. Sarah enroule le ruban autour d'un doigt. Chaque tour compte un rayon, sans tirer Nino. La craie s'arrête, et le bleu se desserre. Mon &lt;emphasis&gt;soleil&lt;/emphasis&gt; est rond, comme ta boucle. Tu viens, alors ? Oui, j'apporte la craie. Tu as laissé le soleil finir. [pause]</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -13384,11 +13382,11 @@
       <c r="AW66" t="inlineStr">
         <is>
           <t>enfant-f|J'attends le dernier trait.
-copain|Merci, Sarah.
-narrateur|Elle compte les rayons sur le ruban bleu.
-narrateur|Le ruban attend à la branche, vide.
-narrateur|La craie s'arrête, pile.
-copain|Il a son soleil, là.
+copain|Merci, ta boucle après.
+narrateur|Sarah enroule le ruban autour d'un doigt.
+narrateur|Chaque tour compte un rayon, sans tirer Nino.
+narrateur|La craie s'arrête, et le bleu se desserre.
+copain|Mon soleil est rond, comme ta boucle.
 enfant-f|Tu viens, alors ?
 copain|Oui, j'apporte la craie.
 papa|Tu as laissé le soleil finir.</t>
@@ -13423,17 +13421,17 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Le soleil de craie reste sur la pierre. Il a son dernier trait, Sarah. Oui, tout jaune. La craie a laissé la place. Le prunier fait un petit toc. Le ruban bleu tient un nœud, ferme. Nino glisse le grelot dans la boucle. Le jardin chante, là. Nino pose sa craie au pied du prunier.</t>
+          <t>Le soleil de craie regarde la boucle vide. Il a son dernier trait, Sarah. Oui, bien jaune. La craie a laissé la place. Le prunier fait un petit toc. Le ruban bleu tient un nœud, ferme. Nino glisse le grelot dans la boucle. Le jardin chante, là. Nino pose sa craie au pied du prunier.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le soleil de craie reste sur la pierre. Il a son dernier trait, Sarah. Oui, tout jaune. La craie a laissé la place. Le &lt;emphasis level="moderate"&gt;prunier&lt;/emphasis&gt; fait un petit toc. Le ruban bleu tient un nœud, ferme. Nino glisse le grelot dans la boucle. Le jardin chante, là. Nino pose sa craie au pied du prunier.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le soleil de craie regarde la boucle vide. Il a son dernier trait, Sarah. Oui, bien jaune. La craie a laissé la place. Le &lt;emphasis level="moderate"&gt;prunier&lt;/emphasis&gt; fait un petit toc. Le ruban bleu tient un nœud, ferme. Nino glisse le grelot dans la boucle. Le jardin chante, là. Nino pose sa craie au pied du prunier.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le soleil de craie reste sur la pierre. Il a son dernier trait, Sarah. Oui, tout jaune. La craie a laissé la place. Le &lt;emphasis&gt;prunier&lt;/emphasis&gt; fait un petit toc. Le ruban bleu tient un nœud, ferme. Nino glisse le grelot dans la boucle. Le jardin chante, là. Nino pose sa craie au pied du prunier.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le soleil de craie regarde la boucle vide. Il a son dernier trait, Sarah. Oui, bien jaune. La craie a laissé la place. Le &lt;emphasis&gt;prunier&lt;/emphasis&gt; fait un petit toc. Le ruban bleu tient un nœud, ferme. Nino glisse le grelot dans la boucle. Le jardin chante, là. Nino pose sa craie au pied du prunier.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
@@ -13571,9 +13569,9 @@
       </c>
       <c r="AW67" t="inlineStr">
         <is>
-          <t>narrateur|Le soleil de craie reste sur la pierre.
+          <t>narrateur|Le soleil de craie regarde la boucle vide.
 copain|Il a son dernier trait, Sarah.
-enfant-f|Oui, tout jaune.
+enfant-f|Oui, bien jaune.
 papa|La craie a laissé la place.
 maman|Le prunier fait un petit toc.
 narrateur|Le ruban bleu tient un nœud, ferme.
@@ -13611,17 +13609,17 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Nino, un carillon t'écoute. Elle montre la boucle, de loin, sans crier. Sa voix reste près de lui, presque un souffle. Il a une oreille, lui aussi ? Oui, bleue comme le ciel. Je viens, alors. Il pose la craie, sans la perdre. Tu as parlé contre son dessin. C'est lui qui a dit oui.</t>
+          <t>Nino, la boucle t'écoute, de loin. Elle montre le bleu, sans quitter la terrasse. Sa voix reste un souffle, collée à la craie. Elle a une oreille, la branche ? Oui, bleue comme le ciel. Je viens, alors. Il pose la craie, et suit le ruban des yeux. Tu as parlé contre son dessin. C'est lui qui a dit oui.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino, un &lt;emphasis level="moderate"&gt;carillon&lt;/emphasis&gt; t'écoute. Elle montre la boucle, de loin, sans crier. Sa voix reste près de lui, presque un souffle. Il a une oreille, lui aussi ? Oui, bleue comme le ciel. Je viens, alors. Il pose la craie, sans la perdre. Tu as parlé contre son dessin. C'est lui qui a dit oui.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino, la boucle t'écoute, de loin. Elle montre le bleu, sans quitter la terrasse. Sa voix reste un souffle, collée à la craie. Elle a une oreille, la branche ? Oui, bleue comme le ciel. Je viens, alors. Il pose la craie, et suit le ruban des yeux. Tu as parlé contre son dessin. C'est lui qui a dit oui.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Nino, un &lt;emphasis&gt;carillon&lt;/emphasis&gt; t'écoute. Elle montre la boucle, de loin, sans crier. Sa voix reste près de lui, presque un souffle. Il a une oreille, lui aussi ? Oui, bleue comme le ciel. Je viens, alors. Il pose la craie, sans la perdre. Tu as parlé contre son dessin. C'est lui qui a dit oui. [pause]</t>
+          <t>Nino, la boucle t'écoute, de loin. Elle montre le bleu, sans quitter la terrasse. Sa voix reste un souffle, collée à la craie. Elle a une oreille, la branche ? Oui, bleue comme le ciel. Je viens, alors. Il pose la craie, et suit le ruban des yeux. Tu as parlé contre son dessin. C'est lui qui a dit oui. [pause]</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -13755,13 +13753,13 @@
       </c>
       <c r="AW68" t="inlineStr">
         <is>
-          <t>enfant-f|Nino, un carillon t'écoute.
-narrateur|Elle montre la boucle, de loin, sans crier.
-narrateur|Sa voix reste près de lui, presque un souffle.
-copain|Il a une oreille, lui aussi ?
+          <t>enfant-f|Nino, la boucle t'écoute, de loin.
+narrateur|Elle montre le bleu, sans quitter la terrasse.
+narrateur|Sa voix reste un souffle, collée à la craie.
+copain|Elle a une oreille, la branche ?
 enfant-f|Oui, bleue comme le ciel.
 copain|Je viens, alors.
-narrateur|Il pose la craie, sans la perdre.
+narrateur|Il pose la craie, et suit le ruban des yeux.
 papa|Tu as parlé contre son dessin.
 maman|C'est lui qui a dit oui.</t>
         </is>
@@ -13983,17 +13981,17 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Je m'assois à côté. Sarah s'assoit dans l'herbe, sous la branche. Elle ne touche pas la craie. Tu vois le rayon, toi aussi ? Oui, il pique un peu. Un dernier trait les fait souffler. On accroche, après ça. Tu as écouté son soleil. C'est lui qui a dit après.</t>
+          <t>Je m'assois à côté. Sarah s'assoit dans l'herbe, sous la branche. Le ruban lui fait un bracelet, un peu rêche. Tu vois le rayon, toi aussi ? Oui, il pique un peu. Un dernier trait les fait souffler ensemble. On accroche, après ça. Tu as écouté son soleil. C'est lui qui a dit après.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Je m'assois à &lt;emphasis level="moderate"&gt;côté&lt;/emphasis&gt;. Sarah s'assoit dans l'herbe, sous la branche. Elle ne touche pas la craie. Tu vois le rayon, toi aussi ? Oui, il pique un peu. Un dernier trait les fait souffler. On accroche, après ça. Tu as écouté son soleil. C'est lui qui a dit après.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Je m'assois à &lt;emphasis level="moderate"&gt;côté&lt;/emphasis&gt;. Sarah s'assoit dans l'herbe, sous la branche. Le ruban lui fait un bracelet, un peu rêche. Tu vois le rayon, toi aussi ? Oui, il pique un peu. Un dernier trait les fait souffler ensemble. On accroche, après ça. Tu as écouté son soleil. C'est lui qui a dit après.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Je m'assois à &lt;emphasis&gt;côté&lt;/emphasis&gt;. Sarah s'assoit dans l'herbe, sous la branche. Elle ne touche pas la craie. Tu vois le rayon, toi aussi ? Oui, il pique un peu. Un dernier trait les fait souffler. On accroche, après ça. Tu as écouté son soleil. C'est lui qui a dit après. [pause]</t>
+          <t>Je m'assois à &lt;emphasis&gt;côté&lt;/emphasis&gt;. Sarah s'assoit dans l'herbe, sous la branche. Le ruban lui fait un bracelet, un peu rêche. Tu vois le rayon, toi aussi ? Oui, il pique un peu. Un dernier trait les fait souffler ensemble. On accroche, après ça. Tu as écouté son soleil. C'est lui qui a dit après. [pause]</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr"/>
@@ -14129,10 +14127,10 @@
         <is>
           <t>enfant-f|Je m'assois à côté.
 narrateur|Sarah s'assoit dans l'herbe, sous la branche.
-narrateur|Elle ne touche pas la craie.
+narrateur|Le ruban lui fait un bracelet, un peu rêche.
 copain|Tu vois le rayon, toi aussi ?
 enfant-f|Oui, il pique un peu.
-narrateur|Un dernier trait les fait souffler.
+narrateur|Un dernier trait les fait souffler ensemble.
 copain|On accroche, après ça.
 papa|Tu as écouté son soleil.
 maman|C'est lui qui a dit après.</t>
@@ -14355,17 +14353,17 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Sarah quitte la branche, le ruban en place. Nino respire contre la rose, tout entier. Nino, ma boucle t'attend. Elle n'a pas volé. Tu viens sous le prunier ? La coccinelle, d'abord. Une patte rouge reste collée, immobile. Sarah baisse les yeux, un peu seule. Il ne veut pas bouger. Tu fais quoi, alors ?</t>
+          <t>Sarah quitte la branche, le ruban en place. Nino respire contre la rose, jusqu'aux épaules. Nino, ma boucle t'attend. Elle n'a pas volé. Tu viens sous le prunier ? La coccinelle, d'abord. Une patte rouge reste collée, immobile. Sarah baisse les yeux, un peu seule. Il ne veut pas bouger. Tu fais quoi, alors ?</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Sarah quitte la branche, le ruban en place. Nino respire contre la rose, tout entier. Nino, ma boucle t'attend. Elle n'a pas volé. Tu viens sous le prunier ? La &lt;emphasis level="moderate"&gt;coccinelle&lt;/emphasis&gt;, d'abord. Une patte rouge reste collée, immobile. Sarah baisse les yeux, un peu seule. Il ne veut pas bouger. Tu fais quoi, alors ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Sarah quitte la branche, le ruban en place. Nino respire contre la rose, jusqu'aux épaules. Nino, ma boucle t'attend. Elle n'a pas volé. Tu viens sous le prunier ? La &lt;emphasis level="moderate"&gt;coccinelle&lt;/emphasis&gt;, d'abord. Une patte rouge reste collée, immobile. Sarah baisse les yeux, un peu seule. Il ne veut pas bouger. Tu fais quoi, alors ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Sarah quitte la branche, le ruban en place. Nino respire contre la rose, tout entier. Nino, ma boucle t'attend. Elle n'a pas volé. Tu viens sous le prunier ? La &lt;emphasis&gt;coccinelle&lt;/emphasis&gt;, d'abord. Une patte rouge reste collée, immobile. Sarah baisse les yeux, un peu seule. Il ne veut pas bouger. Tu fais quoi, alors ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Sarah quitte la branche, le ruban en place. Nino respire contre la rose, jusqu'aux épaules. Nino, ma boucle t'attend. Elle n'a pas volé. Tu viens sous le prunier ? La &lt;emphasis&gt;coccinelle&lt;/emphasis&gt;, d'abord. Une patte rouge reste collée, immobile. Sarah baisse les yeux, un peu seule. Il ne veut pas bouger. Tu fais quoi, alors ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
@@ -14504,7 +14502,7 @@
       <c r="AW72" t="inlineStr">
         <is>
           <t>narrateur|Sarah quitte la branche, le ruban en place.
-narrateur|Nino respire contre la rose, tout entier.
+narrateur|Nino respire contre la rose, jusqu'aux épaules.
 enfant-f|Nino, ma boucle t'attend.
 copain|Elle n'a pas volé.
 enfant-f|Tu viens sous le prunier ?
@@ -14740,17 +14738,17 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>J'attends l'envol. Merci, Sarah. La branche garde sa boucle, vide. La coccinelle ouvre une aile, puis part. Elle a volé, là. Tu viens, alors ? Oui, je laisse la rose. Tu as laissé la rose finir. Il a dit oui, après.</t>
+          <t>J'attends l'envol. Merci, pas de boucle trop près. Sarah laisse le ruban à la branche, loin de la rose. La petite bête n'a que le souffle de Nino. Une aile s'ouvre, et l'hôte quitte la fleur. Elle a volé, là. Tu viens, alors ? Oui, je laisse la rose. Tu as laissé la rose finir.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'attends l'&lt;emphasis level="moderate"&gt;envol&lt;/emphasis&gt;. Merci, Sarah. La branche garde sa boucle, vide. La coccinelle ouvre une aile, puis part. Elle a volé, là. Tu viens, alors ? Oui, je laisse la rose. Tu as laissé la rose finir. Il a dit oui, après.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'attends l'&lt;emphasis level="moderate"&gt;envol&lt;/emphasis&gt;. Merci, pas de boucle trop près. Sarah laisse le ruban à la branche, loin de la rose. La petite bête n'a que le souffle de Nino. Une aile s'ouvre, et l'hôte quitte la fleur. Elle a volé, là. Tu viens, alors ? Oui, je laisse la rose. Tu as laissé la rose finir.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>J'attends l'&lt;emphasis&gt;envol&lt;/emphasis&gt;. Merci, Sarah. La branche garde sa boucle, vide. La coccinelle ouvre une aile, puis part. Elle a volé, là. Tu viens, alors ? Oui, je laisse la rose. Tu as laissé la rose finir. Il a dit oui, après. [pause]</t>
+          <t>J'attends l'&lt;emphasis&gt;envol&lt;/emphasis&gt;. Merci, pas de boucle trop près. Sarah laisse le ruban à la branche, loin de la rose. La petite bête n'a que le souffle de Nino. Une aile s'ouvre, et l'hôte quitte la fleur. Elle a volé, là. Tu viens, alors ? Oui, je laisse la rose. Tu as laissé la rose finir. [pause]</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
@@ -14885,14 +14883,14 @@
       <c r="AW74" t="inlineStr">
         <is>
           <t>enfant-f|J'attends l'envol.
-copain|Merci, Sarah.
-narrateur|La branche garde sa boucle, vide.
-narrateur|La coccinelle ouvre une aile, puis part.
+copain|Merci, pas de boucle trop près.
+narrateur|Sarah laisse le ruban à la branche, loin de la rose.
+narrateur|La petite bête n'a que le souffle de Nino.
+narrateur|Une aile s'ouvre, et l'hôte quitte la fleur.
 copain|Elle a volé, là.
 enfant-f|Tu viens, alors ?
 copain|Oui, je laisse la rose.
-papa|Tu as laissé la rose finir.
-maman|Il a dit oui, après.</t>
+papa|Tu as laissé la rose finir.</t>
         </is>
       </c>
       <c r="AX74" t="inlineStr">
@@ -14924,17 +14922,17 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>La rose est vide, à présent. Elle a volé, Sarah. Tu as dit oui, après. Les ailes se sont tues. Le grelot glisse vers la branche. Le ruban bleu tient un nœud, ferme. Nino souffle sur la boucle, minuscule. Il chante, dans le bleu. Le ruban bat, et la rose n'a plus d'hôte.</t>
+          <t>La rose est vide, et le bleu bat un peu. Elle a volé, Sarah. Tu as dit oui, après. Les ailes se sont tues. Le grelot glisse vers la branche. Le ruban bleu tient un nœud, ferme. Nino souffle sur la boucle, minuscule. Il chante, dans le bleu. Le ruban bat, et la rose n'a plus d'hôte.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La rose est vide, à présent. Elle a volé, Sarah. Tu as dit oui, après. Les ailes se sont tues. Le grelot glisse vers la branche. Le ruban bleu tient un nœud, ferme. Nino souffle sur la boucle, minuscule. Il chante, dans le bleu. Le ruban bat, et la rose n'a plus d'hôte.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La rose est vide, et le bleu bat un peu. Elle a volé, Sarah. Tu as dit oui, après. Les ailes se sont tues. Le grelot glisse vers la branche. Le ruban bleu tient un nœud, ferme. Nino souffle sur la boucle, minuscule. Il chante, dans le bleu. Le ruban bat, et la rose n'a plus d'hôte.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La rose est vide, à présent. Elle a volé, Sarah. Tu as dit oui, après. Les ailes se sont tues. Le grelot glisse vers la branche. Le ruban bleu tient un nœud, ferme. Nino souffle sur la boucle, minuscule. Il chante, dans le bleu. Le ruban bat, et la rose n'a plus d'hôte.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La rose est vide, et le bleu bat un peu. Elle a volé, Sarah. Tu as dit oui, après. Les ailes se sont tues. Le grelot glisse vers la branche. Le ruban bleu tient un nœud, ferme. Nino souffle sur la boucle, minuscule. Il chante, dans le bleu. Le ruban bat, et la rose n'a plus d'hôte.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr"/>
@@ -15072,7 +15070,7 @@
       </c>
       <c r="AW75" t="inlineStr">
         <is>
-          <t>narrateur|La rose est vide, à présent.
+          <t>narrateur|La rose est vide, et le bleu bat un peu.
 copain|Elle a volé, Sarah.
 enfant-f|Tu as dit oui, après.
 papa|Les ailes se sont tues.
@@ -15112,17 +15110,17 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Nino, un grelot minuscule ? Elle agite le ruban, une seconde seulement. Elle l'entend, la petite ? Bas, oui. Une aile se lève, puis se rassoit. On va jusqu'au prunier, alors. D'accord. Le son n'a pas chassé la rose. Il a choisi le voyage.</t>
+          <t>Nino, un bleu minuscule ? Elle agite le ruban, une seconde seulement. Elle l'entend, la petite ? Bas, oui. Une aile se lève, puis se rassoit sur le bleu. On va jusqu'au prunier, alors. D'accord. Le tissu n'a pas chassé la rose. Il a choisi le voyage.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino, un &lt;emphasis level="moderate"&gt;grelot&lt;/emphasis&gt; minuscule ? Elle agite le ruban, une seconde seulement. Elle l'entend, la petite ? Bas, oui. Une aile se lève, puis se rassoit. On va jusqu'au prunier, alors. D'accord. Le son n'a pas chassé la rose. Il a choisi le voyage.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino, un bleu minuscule ? Elle agite le ruban, une seconde seulement. Elle l'entend, la petite ? Bas, oui. Une aile se lève, puis se rassoit sur le bleu. On va jusqu'au prunier, alors. D'accord. Le tissu n'a pas chassé la rose. Il a choisi le voyage.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Nino, un &lt;emphasis&gt;grelot&lt;/emphasis&gt; minuscule ? Elle agite le ruban, une seconde seulement. Elle l'entend, la petite ? Bas, oui. Une aile se lève, puis se rassoit. On va jusqu'au prunier, alors. D'accord. Le son n'a pas chassé la rose. Il a choisi le voyage. [pause]</t>
+          <t>Nino, un bleu minuscule ? Elle agite le ruban, une seconde seulement. Elle l'entend, la petite ? Bas, oui. Une aile se lève, puis se rassoit sur le bleu. On va jusqu'au prunier, alors. D'accord. Le tissu n'a pas chassé la rose. Il a choisi le voyage. [pause]</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -15256,14 +15254,14 @@
       </c>
       <c r="AW76" t="inlineStr">
         <is>
-          <t>enfant-f|Nino, un grelot minuscule ?
+          <t>enfant-f|Nino, un bleu minuscule ?
 narrateur|Elle agite le ruban, une seconde seulement.
 copain|Elle l'entend, la petite ?
 enfant-f|Bas, oui.
-narrateur|Une aile se lève, puis se rassoit.
+narrateur|Une aile se lève, puis se rassoit sur le bleu.
 copain|On va jusqu'au prunier, alors.
 enfant-f|D'accord.
-papa|Le son n'a pas chassé la rose.
+papa|Le tissu n'a pas chassé la rose.
 maman|Il a choisi le voyage.</t>
         </is>
       </c>
@@ -15484,17 +15482,17 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Pas maintenant, Sarah. D'accord. Elle serre le ruban, les épaules basses. J'accroche ici, alors. Le ruban reste à la branche, à elle. Un battement bleu part vers la rose, loin. Je l'entends, d'ici ! Toi la rose, moi le prunier. Tu as gardé ton carillon. La rose est restée à lui.</t>
+          <t>Pas maintenant, Sarah. D'accord. Elle serre le ruban, les épaules basses. J'accroche à la branche, alors. Un battement bleu part vers la rose, loin. Je l'entends, d'ici ! Toi la rose, moi le nœud. Tu as gardé ton carillon. La rose est restée à lui.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Pas maintenant, Sarah. D'accord. Elle serre le ruban, les épaules basses. J'accroche ici, alors. Le ruban reste à la branche, à elle. Un battement bleu part vers la rose, loin. Je l'entends, d'ici ! Toi la rose, moi le prunier. Tu as gardé ton &lt;emphasis level="moderate"&gt;carillon&lt;/emphasis&gt;. La rose est restée à lui.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Pas maintenant, Sarah. D'accord. Elle serre le ruban, les épaules basses. J'accroche à la branche, alors. Un battement bleu part vers la rose, loin. Je l'entends, d'ici ! Toi la rose, moi le nœud. Tu as gardé ton &lt;emphasis level="moderate"&gt;carillon&lt;/emphasis&gt;. La rose est restée à lui.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Pas maintenant, Sarah. D'accord. Elle serre le ruban, les épaules basses. J'accroche ici, alors. Le ruban reste à la branche, à elle. Un battement bleu part vers la rose, loin. Je l'entends, d'ici ! Toi la rose, moi le prunier. Tu as gardé ton &lt;emphasis&gt;carillon&lt;/emphasis&gt;. La rose est restée à lui. [pause]</t>
+          <t>Pas maintenant, Sarah. D'accord. Elle serre le ruban, les épaules basses. J'accroche à la branche, alors. Un battement bleu part vers la rose, loin. Je l'entends, d'ici ! Toi la rose, moi le nœud. Tu as gardé ton &lt;emphasis&gt;carillon&lt;/emphasis&gt;. La rose est restée à lui. [pause]</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
@@ -15631,11 +15629,10 @@
           <t>copain|Pas maintenant, Sarah.
 enfant-f|D'accord.
 narrateur|Elle serre le ruban, les épaules basses.
-enfant-f|J'accroche ici, alors.
-narrateur|Le ruban reste à la branche, à elle.
+enfant-f|J'accroche à la branche, alors.
 narrateur|Un battement bleu part vers la rose, loin.
 copain|Je l'entends, d'ici !
-enfant-f|Toi la rose, moi le prunier.
+enfant-f|Toi la rose, moi le nœud.
 papa|Tu as gardé ton carillon.
 maman|La rose est restée à lui.</t>
         </is>
@@ -16242,17 +16239,17 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>J'aide un peu. Elle fouille sous le prunier, sans se presser. Une sandale chaude apparaît, collée aux prunes. Elle s'était cachée ! Près du bord, oui. Deux pieds, à présent, bien chauds. On peut accrocher, là. Tu as cherché avec lui. Le pied nu n'a plus froid.</t>
+          <t>J'aide un peu. Elle plante le ruban comme un drapeau, sous les prunes. Une sandale chaude apparaît, collée aux fruits. Elle s'était cachée sous le prunier ! Près du bord, oui. Deux pieds, à présent, bien chauds. On peut accrocher, là. Tu as cherché avec lui. Le pied nu n'a plus froid.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'aide un peu. Elle fouille sous le prunier, sans se presser. Une &lt;emphasis level="moderate"&gt;sandale&lt;/emphasis&gt; chaude apparaît, collée aux prunes. Elle s'était cachée ! Près du bord, oui. Deux pieds, à présent, bien chauds. On peut accrocher, là. Tu as cherché avec lui. Le pied nu n'a plus froid.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'aide un peu. Elle plante le ruban comme un drapeau, sous les prunes. Une &lt;emphasis level="moderate"&gt;sandale&lt;/emphasis&gt; chaude apparaît, collée aux fruits. Elle s'était cachée sous le prunier ! Près du bord, oui. Deux pieds, à présent, bien chauds. On peut accrocher, là. Tu as cherché avec lui. Le pied nu n'a plus froid.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>J'aide un peu. Elle fouille sous le prunier, sans se presser. Une &lt;emphasis&gt;sandale&lt;/emphasis&gt; chaude apparaît, collée aux prunes. Elle s'était cachée ! Près du bord, oui. Deux pieds, à présent, bien chauds. On peut accrocher, là. Tu as cherché avec lui. Le pied nu n'a plus froid. [pause]</t>
+          <t>J'aide un peu. Elle plante le ruban comme un drapeau, sous les prunes. Une &lt;emphasis&gt;sandale&lt;/emphasis&gt; chaude apparaît, collée aux fruits. Elle s'était cachée sous le prunier ! Près du bord, oui. Deux pieds, à présent, bien chauds. On peut accrocher, là. Tu as cherché avec lui. Le pied nu n'a plus froid. [pause]</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr"/>
@@ -16387,9 +16384,9 @@
       <c r="AW82" t="inlineStr">
         <is>
           <t>enfant-f|J'aide un peu.
-narrateur|Elle fouille sous le prunier, sans se presser.
-narrateur|Une sandale chaude apparaît, collée aux prunes.
-copain|Elle s'était cachée !
+narrateur|Elle plante le ruban comme un drapeau, sous les prunes.
+narrateur|Une sandale chaude apparaît, collée aux fruits.
+copain|Elle s'était cachée sous le prunier !
 enfant-f|Près du bord, oui.
 narrateur|Deux pieds, à présent, bien chauds.
 copain|On peut accrocher, là.
@@ -16426,17 +16423,17 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Les deux sandales sont chaudes, enfin. Le pied nu n'a plus froid. On peut accrocher, là. Vous avez cherché ensemble. La branche attend, un peu. Le ruban bleu tient un nœud, ferme. Nino s'assoit, le pied au chaud. Le carillon est prêt, pour deux. La sandale était sous les prunes, au frais.</t>
+          <t>Les deux sandales fument un peu, sous les prunes. Le pied nu n'a plus froid. On peut accrocher, là. Vous avez cherché ensemble. La branche attend, un peu. Le ruban bleu tient un nœud, ferme. Nino s'assoit, le pied au chaud. Le carillon est prêt, pour deux. La sandale était sous les prunes, au frais.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les deux sandales sont chaudes, enfin. Le pied nu n'a plus froid. On peut accrocher, là. Vous avez cherché ensemble. La branche attend, un peu. Le ruban bleu tient un nœud, ferme. Nino s'assoit, le pied au chaud. Le carillon est prêt, pour deux. La sandale était sous les prunes, au frais.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les deux sandales fument un peu, sous les prunes. Le pied nu n'a plus froid. On peut accrocher, là. Vous avez cherché ensemble. La branche attend, un peu. Le ruban bleu tient un nœud, ferme. Nino s'assoit, le pied au chaud. Le carillon est prêt, pour deux. La sandale était sous les prunes, au frais.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les deux sandales sont chaudes, enfin. Le pied nu n'a plus froid. On peut accrocher, là. Vous avez cherché ensemble. La branche attend, un peu. Le ruban bleu tient un nœud, ferme. Nino s'assoit, le pied au chaud. Le carillon est prêt, pour deux. La sandale était sous les prunes, au frais.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les deux sandales fument un peu, sous les prunes. Le pied nu n'a plus froid. On peut accrocher, là. Vous avez cherché ensemble. La branche attend, un peu. Le ruban bleu tient un nœud, ferme. Nino s'assoit, le pied au chaud. Le carillon est prêt, pour deux. La sandale était sous les prunes, au frais.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -16574,7 +16571,7 @@
       </c>
       <c r="AW83" t="inlineStr">
         <is>
-          <t>narrateur|Les deux sandales sont chaudes, enfin.
+          <t>narrateur|Les deux sandales fument un peu, sous les prunes.
 copain|Le pied nu n'a plus froid.
 enfant-f|On peut accrocher, là.
 papa|Vous avez cherché ensemble.
@@ -16614,17 +16611,17 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Un petit regard, Nino ? Très petit, alors. D'accord. Ils se penchent vers la boucle, une seconde. Un bleu brille, une seconde. Il chante, presque. Puis Nino reprend la sandale. Tu as montré juste un peu. Il a vu, puis choisi.</t>
+          <t>Un petit regard, Nino ? Le temps d'un bleu, alors. D'accord. Nino lève les yeux vers la boucle, une seconde. Le ruban bat, puis se tait. J'ai vu, je cherche. Il baisse la tête, et fouille l'herbe à nouveau. Tu as montré juste un peu. Il a vu, puis choisi.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un petit &lt;emphasis level="moderate"&gt;regard&lt;/emphasis&gt;, Nino ? Très petit, alors. D'accord. Ils se penchent vers la boucle, une seconde. Un bleu brille, une seconde. Il chante, presque. Puis Nino reprend la sandale. Tu as montré juste un peu. Il a vu, puis choisi.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un petit &lt;emphasis level="moderate"&gt;regard&lt;/emphasis&gt;, Nino ? Le temps d'un bleu, alors. D'accord. Nino lève les yeux vers la boucle, une seconde. Le ruban bat, puis se tait. J'ai vu, je cherche. Il baisse la tête, et fouille l'herbe à nouveau. Tu as montré juste un peu. Il a vu, puis choisi.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Un petit &lt;emphasis&gt;regard&lt;/emphasis&gt;, Nino ? Très petit, alors. D'accord. Ils se penchent vers la boucle, une seconde. Un bleu brille, une seconde. Il chante, presque. Puis Nino reprend la sandale. Tu as montré juste un peu. Il a vu, puis choisi. [pause]</t>
+          <t>Un petit &lt;emphasis&gt;regard&lt;/emphasis&gt;, Nino ? Le temps d'un bleu, alors. D'accord. Nino lève les yeux vers la boucle, une seconde. Le ruban bat, puis se tait. J'ai vu, je cherche. Il baisse la tête, et fouille l'herbe à nouveau. Tu as montré juste un peu. Il a vu, puis choisi. [pause]</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
@@ -16759,12 +16756,12 @@
       <c r="AW84" t="inlineStr">
         <is>
           <t>enfant-f|Un petit regard, Nino ?
-copain|Très petit, alors.
+copain|Le temps d'un bleu, alors.
 enfant-f|D'accord.
-narrateur|Ils se penchent vers la boucle, une seconde.
-narrateur|Un bleu brille, une seconde.
-copain|Il chante, presque.
-narrateur|Puis Nino reprend la sandale.
+narrateur|Nino lève les yeux vers la boucle, une seconde.
+narrateur|Le ruban bat, puis se tait.
+copain|J'ai vu, je cherche.
+narrateur|Il baisse la tête, et fouille l'herbe à nouveau.
 papa|Tu as montré juste un peu.
 maman|Il a vu, puis choisi.</t>
         </is>
@@ -16986,17 +16983,17 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>On accroche plus tard, alors ? Oui, plus tard. D'accord. Le prunier garde sa boucle, pour lui. Nino serre la sandale, concentré. Garde un son pour moi. Il t'attend à la branche. Tu as dit une autre heure. Le pied nu cherche, lui.</t>
+          <t>On accroche plus tard, alors ? Oui, plus tard, le pied d'abord. D'accord. Sarah laisse la boucle vide, à la branche. Nino serre la sandale, concentré. Garde un bleu pour moi. Il t'attend à la branche. Tu as dit une autre heure. Le pied nu cherche, lui.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On accroche &lt;emphasis level="moderate"&gt;plus tard&lt;/emphasis&gt;, alors ? Oui, plus tard. D'accord. Le prunier garde sa boucle, pour lui. Nino serre la sandale, concentré. Garde un son pour moi. Il t'attend à la branche. Tu as dit une autre heure. Le pied nu cherche, lui.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On accroche &lt;emphasis level="moderate"&gt;plus tard&lt;/emphasis&gt;, alors ? Oui, plus tard, le pied d'abord. D'accord. Sarah laisse la boucle vide, à la branche. Nino serre la sandale, concentré. Garde un bleu pour moi. Il t'attend à la branche. Tu as dit une autre heure. Le pied nu cherche, lui.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>On accroche &lt;emphasis&gt;plus tard&lt;/emphasis&gt;, alors ? Oui, plus tard. D'accord. Le prunier garde sa boucle, pour lui. Nino serre la sandale, concentré. Garde un son pour moi. Il t'attend à la branche. Tu as dit une autre heure. Le pied nu cherche, lui. [pause]</t>
+          <t>On accroche &lt;emphasis&gt;plus tard&lt;/emphasis&gt;, alors ? Oui, plus tard, le pied d'abord. D'accord. Sarah laisse la boucle vide, à la branche. Nino serre la sandale, concentré. Garde un bleu pour moi. Il t'attend à la branche. Tu as dit une autre heure. Le pied nu cherche, lui. [pause]</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
@@ -17131,11 +17128,11 @@
       <c r="AW86" t="inlineStr">
         <is>
           <t>enfant-f|On accroche plus tard, alors ?
-copain|Oui, plus tard.
+copain|Oui, plus tard, le pied d'abord.
 enfant-f|D'accord.
-narrateur|Le prunier garde sa boucle, pour lui.
+narrateur|Sarah laisse la boucle vide, à la branche.
 narrateur|Nino serre la sandale, concentré.
-copain|Garde un son pour moi.
+copain|Garde un bleu pour moi.
 enfant-f|Il t'attend à la branche.
 papa|Tu as dit une autre heure.
 maman|Le pied nu cherche, lui.</t>
@@ -17352,7 +17349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17416,6 +17413,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>